<commit_message>
Add Q1 analysis: county ranking by source type, checklist item 16, README update
</commit_message>
<xml_diff>
--- a/checklist/data-cleaning-checklist.xlsx
+++ b/checklist/data-cleaning-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ANALYTICS PORTFOLIO\kenya-water-points-data-cleaning\checklist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F93DF36-FBE4-428D-B626-98D708635650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD69D2D-F929-42BC-9B4A-F9AE01145C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D102A980-2931-4E60-A925-C3D13E6742CC}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="103">
   <si>
     <t>Category</t>
   </si>
@@ -136,9 +136,6 @@
     <t>After any fix, everything built on the old values still works and the numbers still add up.</t>
   </si>
   <si>
-    <t>Re-run every diagnostic. Look for #REF! errors, formulas searching for text you've since replaced, and SUM ranges that include the wrong rows. Check that any tier counts (for example clean, one issue, multiple issues) add up to the total number of rows.</t>
-  </si>
-  <si>
     <t>Any error, or any count that moved unexpectedly, means something depended on the old data. Explain every changed number before you trust it.</t>
   </si>
   <si>
@@ -317,6 +314,27 @@
   </si>
   <si>
     <t>A client can read the log and understand what you did and why.By the end of a run, every log row has one of four outcomes: fixed, flagged, left unchanged (with the reason), or an open question for the data owner. Nothing should still read "to be decided".</t>
+  </si>
+  <si>
+    <t>A key measure behaves the same way across every source or contributor, with no source that never varies.</t>
+  </si>
+  <si>
+    <t>Break the key measure down by source or contributor with a COUNTIFS table. Look for sources at exactly 0% or 100%, and test them against a related column (for example status_clean against status_id).</t>
+  </si>
+  <si>
+    <t>Similar sources should give similar results. A source at exactly 100% or 0% across hundreds of rows is probably a default or a different way of recording, not a measurement.</t>
+  </si>
+  <si>
+    <t>Don't merge such sources into a headline figure. Report them separately or leave them out, say which, and ask the data owner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Detect </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Break the key measure down by source</t>
+  </si>
+  <si>
+    <t>Re-run every diagnostic. Look for #REF! errors, formulas searching for text you've since replaced, and SUM ranges that include the wrong rows. Check that any tier counts (for example clean, one issue, multiple issues) add up to the total number of rows. Refer to columns by name in logs and notes, not by letter: deleting columns shifts the letters, and a formula typed with an old letter points at the wrong column.</t>
   </si>
 </sst>
 </file>
@@ -674,13 +692,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB2538F-BB86-4D0B-80FA-2C9BD0C63863}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="6.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" customWidth="1"/>
-    <col min="4" max="4" width="36.6640625" customWidth="1"/>
-    <col min="5" max="5" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.88671875" customWidth="1"/>
+    <col min="4" max="4" width="42.44140625" customWidth="1"/>
+    <col min="5" max="5" width="36.44140625" customWidth="1"/>
     <col min="6" max="6" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -716,7 +735,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
@@ -736,10 +755,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -753,10 +772,10 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -796,13 +815,13 @@
         <v>19</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="F6" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
@@ -816,13 +835,13 @@
         <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
@@ -885,7 +904,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -896,13 +915,13 @@
         <v>35</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -910,19 +929,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="72" x14ac:dyDescent="0.3">
@@ -930,19 +949,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
@@ -950,19 +969,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="144" x14ac:dyDescent="0.3">
@@ -970,19 +989,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
@@ -990,20 +1009,49 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>59</v>
-      </c>
+    </row>
+    <row r="17" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1012,26 +1060,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE3BF7B1-7757-49D4-9701-BEBA7F59562E}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" customWidth="1"/>
+    <col min="4" max="4" width="33.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1042,10 +1090,10 @@
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1056,10 +1104,10 @@
         <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1070,10 +1118,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1084,10 +1132,10 @@
         <v>13</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1098,10 +1146,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1112,10 +1160,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1126,10 +1174,10 @@
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1140,10 +1188,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1154,10 +1202,10 @@
         <v>6</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1168,10 +1216,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1182,10 +1230,10 @@
         <v>2</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1196,52 +1244,66 @@
         <v>15</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" s="2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2">
+        <v>10</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B17" s="2">
         <v>9</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>